<commit_message>
feat(customers): allow entering multiple contact personnel per company in form and Excel template
</commit_message>
<xml_diff>
--- a/docs/templates/MERCON_Customers_Import_Template.xlsx
+++ b/docs/templates/MERCON_Customers_Import_Template.xlsx
@@ -12,12 +12,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="75">
   <si>
     <t>🏢 MERCON LOGISTICS  |  ENTERPRISE CUSTOMER ONBOARDING SPECIFICATION</t>
   </si>
   <si>
-    <t>Official onboarding worksheet for Customer Accounts &amp; Commercial Onboarding. Follow instructions below before returning the file.</t>
+    <t>Official onboarding worksheet for Customer Accounts &amp; Commercial Personnel. Follow instructions below before returning the file.</t>
   </si>
   <si>
     <t xml:space="preserve">STATUS
@@ -28,8 +28,8 @@
 Marked with Red Asterisk (*)</t>
   </si>
   <si>
-    <t xml:space="preserve">SUPPORT &amp; INGESTION
-support@mercon-logistics.com</t>
+    <t xml:space="preserve">MULTIPLE CONTACTS
+Enter Primary &amp; Secondary Contacts per Row</t>
   </si>
   <si>
     <t>➊ STEP 1: REVIEW REQUIRED COLUMNS</t>
@@ -38,10 +38,10 @@
     <t>• Columns with a red label and asterisk (*) are MANDATORY for importing.</t>
   </si>
   <si>
-    <t>• Required Customer fields: Company Name *, Primary Phone *.</t>
-  </si>
-  <si>
-    <t>• Optional fields: Trade Name, Industry, Commercial Reg. (CR) No., VAT / Tax Number, Billing Email, Contact Person, Job Title, Address / Notes.</t>
+    <t>• Required Customer fields: Company Name *, Primary Contact Phone *.</t>
+  </si>
+  <si>
+    <t>• Multiple Personnel: Enter Primary Contact details (Name, Phone, Email, Title) and Secondary Contact details (Name, Phone, Email, Title).</t>
   </si>
   <si>
     <t>➋ STEP 2: FILL OUT THE CUSTOMERS DIRECTORY TAB</t>
@@ -50,15 +50,15 @@
     <t>• Switch to the "🏢 Customers Directory" sheet tab at the bottom to enter customer records.</t>
   </si>
   <si>
-    <t>🏢 CUSTOMER ACCOUNTS DIRECTORY  —  BULK DATA ENTRY</t>
+    <t>🏢 CUSTOMER ACCOUNTS DIRECTORY  —  MULTIPLE CONTACT PERSONNEL ENTRY</t>
   </si>
   <si>
     <t xml:space="preserve">MODULE
 Commercial &amp; Customer Directory</t>
   </si>
   <si>
-    <t xml:space="preserve">PRIMARY KEY &amp; CONTACT
-Company Name &amp; Primary Contact Phone</t>
+    <t xml:space="preserve">MULTIPLE PERSONNEL PER COMPANY
+Primary &amp; Secondary Representatives Supported</t>
   </si>
   <si>
     <t xml:space="preserve">INITIAL STATUS
@@ -83,16 +83,28 @@
     <t>VAT / Tax Number</t>
   </si>
   <si>
+    <t>Primary Contact Name</t>
+  </si>
+  <si>
     <t>Primary Phone *</t>
   </si>
   <si>
-    <t>Billing Email</t>
-  </si>
-  <si>
-    <t>Contact Representative</t>
-  </si>
-  <si>
-    <t>Job Title</t>
+    <t>Primary Email</t>
+  </si>
+  <si>
+    <t>Primary Contact Title</t>
+  </si>
+  <si>
+    <t>Secondary Contact Name</t>
+  </si>
+  <si>
+    <t>Secondary Phone</t>
+  </si>
+  <si>
+    <t>Secondary Email</t>
+  </si>
+  <si>
+    <t>Secondary Contact Title</t>
   </si>
   <si>
     <t>Billing Address / Notes</t>
@@ -116,18 +128,30 @@
     <t>310123456700003</t>
   </si>
   <si>
+    <t>Eng. Tariq Al-Mansoor</t>
+  </si>
+  <si>
     <t>+966 50 123 4567</t>
   </si>
   <si>
-    <t>billing@sabic.com</t>
-  </si>
-  <si>
-    <t>Eng. Tariq Al-Mansoor</t>
+    <t>tariq@sabic.com</t>
   </si>
   <si>
     <t>VP of Supply Chain</t>
   </si>
   <si>
+    <t>Sami Al-Otaibi</t>
+  </si>
+  <si>
+    <t>+966 50 123 9999</t>
+  </si>
+  <si>
+    <t>sami@sabic.com</t>
+  </si>
+  <si>
+    <t>Dispatch Ops Lead</t>
+  </si>
+  <si>
     <t>Building 829, King Fahd Road, Riyadh</t>
   </si>
   <si>
@@ -149,18 +173,30 @@
     <t>310987654300003</t>
   </si>
   <si>
+    <t>Fahad Al-Zahrani</t>
+  </si>
+  <si>
     <t>+966 50 987 6543</t>
   </si>
   <si>
-    <t>commercial@almarai.com</t>
-  </si>
-  <si>
-    <t>Fahad Al-Zahrani</t>
+    <t>fahad@almarai.com</t>
   </si>
   <si>
     <t>Logistics Director</t>
   </si>
   <si>
+    <t>Noura Al-Hassan</t>
+  </si>
+  <si>
+    <t>+966 50 987 8888</t>
+  </si>
+  <si>
+    <t>noura@almarai.com</t>
+  </si>
+  <si>
+    <t>Billing Specialist</t>
+  </si>
+  <si>
     <t>Exit 7, Northern Ring Road, Riyadh</t>
   </si>
   <si>
@@ -182,16 +218,28 @@
     <t>310554433200003</t>
   </si>
   <si>
+    <t>Mona Hassan</t>
+  </si>
+  <si>
     <t>+966 55 443 2211</t>
   </si>
   <si>
-    <t>invoicing@panda.com.sa</t>
-  </si>
-  <si>
-    <t>Mona Hassan</t>
-  </si>
-  <si>
-    <t>Procurement Specialist</t>
+    <t>mona@panda.com.sa</t>
+  </si>
+  <si>
+    <t>Procurement Manager</t>
+  </si>
+  <si>
+    <t>Youssef Amer</t>
+  </si>
+  <si>
+    <t>+966 55 443 7777</t>
+  </si>
+  <si>
+    <t>youssef@panda.com.sa</t>
+  </si>
+  <si>
+    <t>Warehouse Manager</t>
   </si>
   <si>
     <t>Al-Andalus District, Jeddah</t>
@@ -870,7 +918,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:K30"/>
+  <dimension ref="A1:O30"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -878,15 +926,18 @@
     <col min="3" max="3" width="22" customWidth="1"/>
     <col min="4" max="4" width="20" customWidth="1"/>
     <col min="5" max="5" width="24" customWidth="1"/>
-    <col min="6" max="6" width="26" customWidth="1"/>
-    <col min="7" max="7" width="24" customWidth="1"/>
-    <col min="8" max="8" width="28" customWidth="1"/>
-    <col min="9" max="9" width="26" customWidth="1"/>
+    <col min="6" max="7" width="26" customWidth="1"/>
+    <col min="8" max="8" width="24" customWidth="1"/>
+    <col min="9" max="9" width="28" customWidth="1"/>
     <col min="10" max="10" width="24" customWidth="1"/>
-    <col min="11" max="11" width="36" customWidth="1"/>
+    <col min="11" max="11" width="26" customWidth="1"/>
+    <col min="12" max="12" width="24" customWidth="1"/>
+    <col min="13" max="13" width="28" customWidth="1"/>
+    <col min="14" max="14" width="24" customWidth="1"/>
+    <col min="15" max="15" width="36" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
         <v>11</v>
       </c>
@@ -900,8 +951,12 @@
       <c r="I1" s="8"/>
       <c r="J1" s="8"/>
       <c r="K1" s="8"/>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L1" s="8"/>
+      <c r="M1" s="8"/>
+      <c r="N1" s="8"/>
+      <c r="O1" s="8"/>
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" s="8"/>
       <c r="B2" s="8"/>
       <c r="C2" s="8"/>
@@ -913,27 +968,35 @@
       <c r="I2" s="8"/>
       <c r="J2" s="8"/>
       <c r="K2" s="8"/>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L2" s="8"/>
+      <c r="M2" s="8"/>
+      <c r="N2" s="8"/>
+      <c r="O2" s="8"/>
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
         <v>12</v>
       </c>
       <c r="B4" s="9"/>
       <c r="C4" s="9"/>
-      <c r="D4" s="9" t="s">
+      <c r="D4" s="9"/>
+      <c r="E4" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="E4" s="9"/>
       <c r="F4" s="9"/>
       <c r="G4" s="9"/>
-      <c r="H4" s="9" t="s">
-        <v>14</v>
-      </c>
+      <c r="H4" s="9"/>
       <c r="I4" s="9"/>
       <c r="J4" s="9"/>
-      <c r="K4" s="9"/>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="K4" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="L4" s="9"/>
+      <c r="M4" s="9"/>
+      <c r="N4" s="9"/>
+      <c r="O4" s="9"/>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5" s="9"/>
       <c r="B5" s="9"/>
       <c r="C5" s="9"/>
@@ -945,8 +1008,12 @@
       <c r="I5" s="9"/>
       <c r="J5" s="9"/>
       <c r="K5" s="9"/>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L5" s="9"/>
+      <c r="M5" s="9"/>
+      <c r="N5" s="9"/>
+      <c r="O5" s="9"/>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7" s="10" t="s">
         <v>15</v>
       </c>
@@ -965,10 +1032,10 @@
       <c r="F7" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="G7" s="11" t="s">
+      <c r="G7" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="H7" s="10" t="s">
+      <c r="H7" s="11" t="s">
         <v>22</v>
       </c>
       <c r="I7" s="10" t="s">
@@ -980,113 +1047,161 @@
       <c r="K7" s="10" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L7" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="M7" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="N7" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="O7" s="10" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8" s="12" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="B8" s="12" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="C8" s="12" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="D8" s="12" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="E8" s="12" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="F8" s="12" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="G8" s="12" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="H8" s="12" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="I8" s="12" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="J8" s="12" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="K8" s="12" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+        <v>40</v>
+      </c>
+      <c r="L8" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="M8" s="12" t="s">
+        <v>42</v>
+      </c>
+      <c r="N8" s="12" t="s">
+        <v>43</v>
+      </c>
+      <c r="O8" s="12" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A9" s="12" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="B9" s="12" t="s">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="C9" s="12" t="s">
-        <v>39</v>
+        <v>47</v>
       </c>
       <c r="D9" s="12" t="s">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="E9" s="12" t="s">
-        <v>41</v>
+        <v>49</v>
       </c>
       <c r="F9" s="12" t="s">
-        <v>42</v>
+        <v>50</v>
       </c>
       <c r="G9" s="12" t="s">
-        <v>43</v>
+        <v>51</v>
       </c>
       <c r="H9" s="12" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="I9" s="12" t="s">
-        <v>45</v>
+        <v>53</v>
       </c>
       <c r="J9" s="12" t="s">
-        <v>46</v>
+        <v>54</v>
       </c>
       <c r="K9" s="12" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+        <v>55</v>
+      </c>
+      <c r="L9" s="12" t="s">
+        <v>56</v>
+      </c>
+      <c r="M9" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="N9" s="12" t="s">
+        <v>58</v>
+      </c>
+      <c r="O9" s="12" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A10" s="12" t="s">
-        <v>48</v>
+        <v>60</v>
       </c>
       <c r="B10" s="12" t="s">
-        <v>49</v>
+        <v>61</v>
       </c>
       <c r="C10" s="12" t="s">
-        <v>50</v>
+        <v>62</v>
       </c>
       <c r="D10" s="12" t="s">
-        <v>51</v>
+        <v>63</v>
       </c>
       <c r="E10" s="12" t="s">
-        <v>52</v>
+        <v>64</v>
       </c>
       <c r="F10" s="12" t="s">
-        <v>53</v>
+        <v>65</v>
       </c>
       <c r="G10" s="12" t="s">
-        <v>54</v>
+        <v>66</v>
       </c>
       <c r="H10" s="12" t="s">
-        <v>55</v>
+        <v>67</v>
       </c>
       <c r="I10" s="12" t="s">
-        <v>56</v>
+        <v>68</v>
       </c>
       <c r="J10" s="12" t="s">
-        <v>57</v>
+        <v>69</v>
       </c>
       <c r="K10" s="12" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+        <v>70</v>
+      </c>
+      <c r="L10" s="12" t="s">
+        <v>71</v>
+      </c>
+      <c r="M10" s="12" t="s">
+        <v>72</v>
+      </c>
+      <c r="N10" s="12" t="s">
+        <v>73</v>
+      </c>
+      <c r="O10" s="12" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A11" s="13"/>
       <c r="B11" s="13"/>
       <c r="C11" s="13"/>
@@ -1098,8 +1213,12 @@
       <c r="I11" s="13"/>
       <c r="J11" s="13"/>
       <c r="K11" s="13"/>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L11" s="13"/>
+      <c r="M11" s="13"/>
+      <c r="N11" s="13"/>
+      <c r="O11" s="13"/>
+    </row>
+    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A12" s="13"/>
       <c r="B12" s="13"/>
       <c r="C12" s="13"/>
@@ -1111,8 +1230,12 @@
       <c r="I12" s="13"/>
       <c r="J12" s="13"/>
       <c r="K12" s="13"/>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L12" s="13"/>
+      <c r="M12" s="13"/>
+      <c r="N12" s="13"/>
+      <c r="O12" s="13"/>
+    </row>
+    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A13" s="13"/>
       <c r="B13" s="13"/>
       <c r="C13" s="13"/>
@@ -1124,8 +1247,12 @@
       <c r="I13" s="13"/>
       <c r="J13" s="13"/>
       <c r="K13" s="13"/>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L13" s="13"/>
+      <c r="M13" s="13"/>
+      <c r="N13" s="13"/>
+      <c r="O13" s="13"/>
+    </row>
+    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A14" s="13"/>
       <c r="B14" s="13"/>
       <c r="C14" s="13"/>
@@ -1137,8 +1264,12 @@
       <c r="I14" s="13"/>
       <c r="J14" s="13"/>
       <c r="K14" s="13"/>
-    </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L14" s="13"/>
+      <c r="M14" s="13"/>
+      <c r="N14" s="13"/>
+      <c r="O14" s="13"/>
+    </row>
+    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A15" s="13"/>
       <c r="B15" s="13"/>
       <c r="C15" s="13"/>
@@ -1150,8 +1281,12 @@
       <c r="I15" s="13"/>
       <c r="J15" s="13"/>
       <c r="K15" s="13"/>
-    </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L15" s="13"/>
+      <c r="M15" s="13"/>
+      <c r="N15" s="13"/>
+      <c r="O15" s="13"/>
+    </row>
+    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A16" s="13"/>
       <c r="B16" s="13"/>
       <c r="C16" s="13"/>
@@ -1163,8 +1298,12 @@
       <c r="I16" s="13"/>
       <c r="J16" s="13"/>
       <c r="K16" s="13"/>
-    </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L16" s="13"/>
+      <c r="M16" s="13"/>
+      <c r="N16" s="13"/>
+      <c r="O16" s="13"/>
+    </row>
+    <row r="17" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A17" s="13"/>
       <c r="B17" s="13"/>
       <c r="C17" s="13"/>
@@ -1176,8 +1315,12 @@
       <c r="I17" s="13"/>
       <c r="J17" s="13"/>
       <c r="K17" s="13"/>
-    </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L17" s="13"/>
+      <c r="M17" s="13"/>
+      <c r="N17" s="13"/>
+      <c r="O17" s="13"/>
+    </row>
+    <row r="18" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A18" s="13"/>
       <c r="B18" s="13"/>
       <c r="C18" s="13"/>
@@ -1189,8 +1332,12 @@
       <c r="I18" s="13"/>
       <c r="J18" s="13"/>
       <c r="K18" s="13"/>
-    </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L18" s="13"/>
+      <c r="M18" s="13"/>
+      <c r="N18" s="13"/>
+      <c r="O18" s="13"/>
+    </row>
+    <row r="19" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A19" s="13"/>
       <c r="B19" s="13"/>
       <c r="C19" s="13"/>
@@ -1202,8 +1349,12 @@
       <c r="I19" s="13"/>
       <c r="J19" s="13"/>
       <c r="K19" s="13"/>
-    </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L19" s="13"/>
+      <c r="M19" s="13"/>
+      <c r="N19" s="13"/>
+      <c r="O19" s="13"/>
+    </row>
+    <row r="20" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A20" s="13"/>
       <c r="B20" s="13"/>
       <c r="C20" s="13"/>
@@ -1215,8 +1366,12 @@
       <c r="I20" s="13"/>
       <c r="J20" s="13"/>
       <c r="K20" s="13"/>
-    </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L20" s="13"/>
+      <c r="M20" s="13"/>
+      <c r="N20" s="13"/>
+      <c r="O20" s="13"/>
+    </row>
+    <row r="21" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A21" s="13"/>
       <c r="B21" s="13"/>
       <c r="C21" s="13"/>
@@ -1228,8 +1383,12 @@
       <c r="I21" s="13"/>
       <c r="J21" s="13"/>
       <c r="K21" s="13"/>
-    </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L21" s="13"/>
+      <c r="M21" s="13"/>
+      <c r="N21" s="13"/>
+      <c r="O21" s="13"/>
+    </row>
+    <row r="22" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A22" s="13"/>
       <c r="B22" s="13"/>
       <c r="C22" s="13"/>
@@ -1241,8 +1400,12 @@
       <c r="I22" s="13"/>
       <c r="J22" s="13"/>
       <c r="K22" s="13"/>
-    </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L22" s="13"/>
+      <c r="M22" s="13"/>
+      <c r="N22" s="13"/>
+      <c r="O22" s="13"/>
+    </row>
+    <row r="23" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A23" s="13"/>
       <c r="B23" s="13"/>
       <c r="C23" s="13"/>
@@ -1254,8 +1417,12 @@
       <c r="I23" s="13"/>
       <c r="J23" s="13"/>
       <c r="K23" s="13"/>
-    </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L23" s="13"/>
+      <c r="M23" s="13"/>
+      <c r="N23" s="13"/>
+      <c r="O23" s="13"/>
+    </row>
+    <row r="24" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A24" s="13"/>
       <c r="B24" s="13"/>
       <c r="C24" s="13"/>
@@ -1267,8 +1434,12 @@
       <c r="I24" s="13"/>
       <c r="J24" s="13"/>
       <c r="K24" s="13"/>
-    </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L24" s="13"/>
+      <c r="M24" s="13"/>
+      <c r="N24" s="13"/>
+      <c r="O24" s="13"/>
+    </row>
+    <row r="25" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A25" s="13"/>
       <c r="B25" s="13"/>
       <c r="C25" s="13"/>
@@ -1280,8 +1451,12 @@
       <c r="I25" s="13"/>
       <c r="J25" s="13"/>
       <c r="K25" s="13"/>
-    </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L25" s="13"/>
+      <c r="M25" s="13"/>
+      <c r="N25" s="13"/>
+      <c r="O25" s="13"/>
+    </row>
+    <row r="26" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A26" s="13"/>
       <c r="B26" s="13"/>
       <c r="C26" s="13"/>
@@ -1293,8 +1468,12 @@
       <c r="I26" s="13"/>
       <c r="J26" s="13"/>
       <c r="K26" s="13"/>
-    </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L26" s="13"/>
+      <c r="M26" s="13"/>
+      <c r="N26" s="13"/>
+      <c r="O26" s="13"/>
+    </row>
+    <row r="27" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A27" s="13"/>
       <c r="B27" s="13"/>
       <c r="C27" s="13"/>
@@ -1306,8 +1485,12 @@
       <c r="I27" s="13"/>
       <c r="J27" s="13"/>
       <c r="K27" s="13"/>
-    </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L27" s="13"/>
+      <c r="M27" s="13"/>
+      <c r="N27" s="13"/>
+      <c r="O27" s="13"/>
+    </row>
+    <row r="28" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A28" s="13"/>
       <c r="B28" s="13"/>
       <c r="C28" s="13"/>
@@ -1319,8 +1502,12 @@
       <c r="I28" s="13"/>
       <c r="J28" s="13"/>
       <c r="K28" s="13"/>
-    </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L28" s="13"/>
+      <c r="M28" s="13"/>
+      <c r="N28" s="13"/>
+      <c r="O28" s="13"/>
+    </row>
+    <row r="29" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A29" s="13"/>
       <c r="B29" s="13"/>
       <c r="C29" s="13"/>
@@ -1332,8 +1519,12 @@
       <c r="I29" s="13"/>
       <c r="J29" s="13"/>
       <c r="K29" s="13"/>
-    </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L29" s="13"/>
+      <c r="M29" s="13"/>
+      <c r="N29" s="13"/>
+      <c r="O29" s="13"/>
+    </row>
+    <row r="30" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A30" s="13"/>
       <c r="B30" s="13"/>
       <c r="C30" s="13"/>
@@ -1345,13 +1536,17 @@
       <c r="I30" s="13"/>
       <c r="J30" s="13"/>
       <c r="K30" s="13"/>
+      <c r="L30" s="13"/>
+      <c r="M30" s="13"/>
+      <c r="N30" s="13"/>
+      <c r="O30" s="13"/>
     </row>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="A1:K2"/>
-    <mergeCell ref="A4:C5"/>
-    <mergeCell ref="D4:G5"/>
-    <mergeCell ref="H4:K5"/>
+    <mergeCell ref="A1:O2"/>
+    <mergeCell ref="A4:D5"/>
+    <mergeCell ref="E4:J5"/>
+    <mergeCell ref="K4:O5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
feat(customers): place contact name and phone side-by-side and add Contact 1, 2, 3 columns to Excel template
</commit_message>
<xml_diff>
--- a/docs/templates/MERCON_Customers_Import_Template.xlsx
+++ b/docs/templates/MERCON_Customers_Import_Template.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="88">
   <si>
     <t>🏢 MERCON LOGISTICS  |  ENTERPRISE CUSTOMER ONBOARDING SPECIFICATION</t>
   </si>
@@ -28,8 +28,8 @@
 Marked with Red Asterisk (*)</t>
   </si>
   <si>
-    <t xml:space="preserve">MULTIPLE CONTACTS
-Enter Primary &amp; Secondary Contacts per Row</t>
+    <t xml:space="preserve">MULTIPLE CONTACT PERSONNEL
+Add Contact 1, Contact 2, Contact 3 per Row</t>
   </si>
   <si>
     <t>➊ STEP 1: REVIEW REQUIRED COLUMNS</t>
@@ -38,10 +38,10 @@
     <t>• Columns with a red label and asterisk (*) are MANDATORY for importing.</t>
   </si>
   <si>
-    <t>• Required Customer fields: Company Name *, Primary Contact Phone *.</t>
-  </si>
-  <si>
-    <t>• Multiple Personnel: Enter Primary Contact details (Name, Phone, Email, Title) and Secondary Contact details (Name, Phone, Email, Title).</t>
+    <t>• Required Customer fields: Company Name *, Contact 1 Phone *.</t>
+  </si>
+  <si>
+    <t>• Multiple Personnel: Enter Contact 1 (Name, Phone, Email, Title), Contact 2 (Name, Phone, Email, Title), and Contact 3 (Name, Phone, Email, Title).</t>
   </si>
   <si>
     <t>➋ STEP 2: FILL OUT THE CUSTOMERS DIRECTORY TAB</t>
@@ -57,8 +57,8 @@
 Commercial &amp; Customer Directory</t>
   </si>
   <si>
-    <t xml:space="preserve">MULTIPLE PERSONNEL PER COMPANY
-Primary &amp; Secondary Representatives Supported</t>
+    <t xml:space="preserve">MULTIPLE CONTACT PERSONNEL PER COMPANY
+Enter Contact 1, Contact 2, Contact 3 side by side</t>
   </si>
   <si>
     <t xml:space="preserve">INITIAL STATUS
@@ -83,28 +83,40 @@
     <t>VAT / Tax Number</t>
   </si>
   <si>
-    <t>Primary Contact Name</t>
-  </si>
-  <si>
-    <t>Primary Phone *</t>
-  </si>
-  <si>
-    <t>Primary Email</t>
-  </si>
-  <si>
-    <t>Primary Contact Title</t>
-  </si>
-  <si>
-    <t>Secondary Contact Name</t>
-  </si>
-  <si>
-    <t>Secondary Phone</t>
-  </si>
-  <si>
-    <t>Secondary Email</t>
-  </si>
-  <si>
-    <t>Secondary Contact Title</t>
+    <t>Contact 1 Name</t>
+  </si>
+  <si>
+    <t>Contact 1 Phone *</t>
+  </si>
+  <si>
+    <t>Contact 1 Email</t>
+  </si>
+  <si>
+    <t>Contact 1 Title</t>
+  </si>
+  <si>
+    <t>Contact 2 Name</t>
+  </si>
+  <si>
+    <t>Contact 2 Phone</t>
+  </si>
+  <si>
+    <t>Contact 2 Email</t>
+  </si>
+  <si>
+    <t>Contact 2 Title</t>
+  </si>
+  <si>
+    <t>Contact 3 Name</t>
+  </si>
+  <si>
+    <t>Contact 3 Phone</t>
+  </si>
+  <si>
+    <t>Contact 3 Email</t>
+  </si>
+  <si>
+    <t>Contact 3 Title</t>
   </si>
   <si>
     <t>Billing Address / Notes</t>
@@ -152,6 +164,18 @@
     <t>Dispatch Ops Lead</t>
   </si>
   <si>
+    <t>Khalid Mansoor</t>
+  </si>
+  <si>
+    <t>+966 50 123 7777</t>
+  </si>
+  <si>
+    <t>khalid@sabic.com</t>
+  </si>
+  <si>
+    <t>Billing Manager</t>
+  </si>
+  <si>
     <t>Building 829, King Fahd Road, Riyadh</t>
   </si>
   <si>
@@ -197,6 +221,18 @@
     <t>Billing Specialist</t>
   </si>
   <si>
+    <t>Salem Al-Harbi</t>
+  </si>
+  <si>
+    <t>+966 50 987 4444</t>
+  </si>
+  <si>
+    <t>salem@almarai.com</t>
+  </si>
+  <si>
+    <t>Fleet Manager</t>
+  </si>
+  <si>
     <t>Exit 7, Northern Ring Road, Riyadh</t>
   </si>
   <si>
@@ -240,6 +276,9 @@
   </si>
   <si>
     <t>Warehouse Manager</t>
+  </si>
+  <si>
+    <t/>
   </si>
   <si>
     <t>Al-Andalus District, Jeddah</t>
@@ -918,7 +957,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:O30"/>
+  <dimension ref="A1:S30"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -934,10 +973,14 @@
     <col min="12" max="12" width="24" customWidth="1"/>
     <col min="13" max="13" width="28" customWidth="1"/>
     <col min="14" max="14" width="24" customWidth="1"/>
-    <col min="15" max="15" width="36" customWidth="1"/>
+    <col min="15" max="15" width="26" customWidth="1"/>
+    <col min="16" max="16" width="24" customWidth="1"/>
+    <col min="17" max="17" width="28" customWidth="1"/>
+    <col min="18" max="18" width="24" customWidth="1"/>
+    <col min="19" max="19" width="36" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
         <v>11</v>
       </c>
@@ -955,8 +998,12 @@
       <c r="M1" s="8"/>
       <c r="N1" s="8"/>
       <c r="O1" s="8"/>
-    </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P1" s="8"/>
+      <c r="Q1" s="8"/>
+      <c r="R1" s="8"/>
+      <c r="S1" s="8"/>
+    </row>
+    <row r="2" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A2" s="8"/>
       <c r="B2" s="8"/>
       <c r="C2" s="8"/>
@@ -972,8 +1019,12 @@
       <c r="M2" s="8"/>
       <c r="N2" s="8"/>
       <c r="O2" s="8"/>
-    </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P2" s="8"/>
+      <c r="Q2" s="8"/>
+      <c r="R2" s="8"/>
+      <c r="S2" s="8"/>
+    </row>
+    <row r="4" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
         <v>12</v>
       </c>
@@ -988,15 +1039,19 @@
       <c r="H4" s="9"/>
       <c r="I4" s="9"/>
       <c r="J4" s="9"/>
-      <c r="K4" s="9" t="s">
-        <v>14</v>
-      </c>
+      <c r="K4" s="9"/>
       <c r="L4" s="9"/>
       <c r="M4" s="9"/>
       <c r="N4" s="9"/>
-      <c r="O4" s="9"/>
-    </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="O4" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="P4" s="9"/>
+      <c r="Q4" s="9"/>
+      <c r="R4" s="9"/>
+      <c r="S4" s="9"/>
+    </row>
+    <row r="5" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A5" s="9"/>
       <c r="B5" s="9"/>
       <c r="C5" s="9"/>
@@ -1012,8 +1067,12 @@
       <c r="M5" s="9"/>
       <c r="N5" s="9"/>
       <c r="O5" s="9"/>
-    </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P5" s="9"/>
+      <c r="Q5" s="9"/>
+      <c r="R5" s="9"/>
+      <c r="S5" s="9"/>
+    </row>
+    <row r="7" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A7" s="10" t="s">
         <v>15</v>
       </c>
@@ -1059,149 +1118,197 @@
       <c r="O7" s="10" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P7" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="Q7" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="R7" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="S7" s="10" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="8" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A8" s="12" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="B8" s="12" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="C8" s="12" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="D8" s="12" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="E8" s="12" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="F8" s="12" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="G8" s="12" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="H8" s="12" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="I8" s="12" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="J8" s="12" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="K8" s="12" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="L8" s="12" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="M8" s="12" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="N8" s="12" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="O8" s="12" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
+        <v>48</v>
+      </c>
+      <c r="P8" s="12" t="s">
+        <v>49</v>
+      </c>
+      <c r="Q8" s="12" t="s">
+        <v>50</v>
+      </c>
+      <c r="R8" s="12" t="s">
+        <v>51</v>
+      </c>
+      <c r="S8" s="12" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="9" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A9" s="12" t="s">
-        <v>45</v>
+        <v>53</v>
       </c>
       <c r="B9" s="12" t="s">
-        <v>46</v>
+        <v>54</v>
       </c>
       <c r="C9" s="12" t="s">
-        <v>47</v>
+        <v>55</v>
       </c>
       <c r="D9" s="12" t="s">
-        <v>48</v>
+        <v>56</v>
       </c>
       <c r="E9" s="12" t="s">
-        <v>49</v>
+        <v>57</v>
       </c>
       <c r="F9" s="12" t="s">
-        <v>50</v>
+        <v>58</v>
       </c>
       <c r="G9" s="12" t="s">
-        <v>51</v>
+        <v>59</v>
       </c>
       <c r="H9" s="12" t="s">
-        <v>52</v>
+        <v>60</v>
       </c>
       <c r="I9" s="12" t="s">
-        <v>53</v>
+        <v>61</v>
       </c>
       <c r="J9" s="12" t="s">
-        <v>54</v>
+        <v>62</v>
       </c>
       <c r="K9" s="12" t="s">
-        <v>55</v>
+        <v>63</v>
       </c>
       <c r="L9" s="12" t="s">
-        <v>56</v>
+        <v>64</v>
       </c>
       <c r="M9" s="12" t="s">
-        <v>57</v>
+        <v>65</v>
       </c>
       <c r="N9" s="12" t="s">
-        <v>58</v>
+        <v>66</v>
       </c>
       <c r="O9" s="12" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
+        <v>67</v>
+      </c>
+      <c r="P9" s="12" t="s">
+        <v>68</v>
+      </c>
+      <c r="Q9" s="12" t="s">
+        <v>69</v>
+      </c>
+      <c r="R9" s="12" t="s">
+        <v>70</v>
+      </c>
+      <c r="S9" s="12" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="10" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A10" s="12" t="s">
-        <v>60</v>
+        <v>72</v>
       </c>
       <c r="B10" s="12" t="s">
-        <v>61</v>
+        <v>73</v>
       </c>
       <c r="C10" s="12" t="s">
-        <v>62</v>
+        <v>74</v>
       </c>
       <c r="D10" s="12" t="s">
-        <v>63</v>
+        <v>75</v>
       </c>
       <c r="E10" s="12" t="s">
-        <v>64</v>
+        <v>76</v>
       </c>
       <c r="F10" s="12" t="s">
-        <v>65</v>
+        <v>77</v>
       </c>
       <c r="G10" s="12" t="s">
-        <v>66</v>
+        <v>78</v>
       </c>
       <c r="H10" s="12" t="s">
-        <v>67</v>
+        <v>79</v>
       </c>
       <c r="I10" s="12" t="s">
-        <v>68</v>
+        <v>80</v>
       </c>
       <c r="J10" s="12" t="s">
-        <v>69</v>
+        <v>81</v>
       </c>
       <c r="K10" s="12" t="s">
-        <v>70</v>
+        <v>82</v>
       </c>
       <c r="L10" s="12" t="s">
-        <v>71</v>
+        <v>83</v>
       </c>
       <c r="M10" s="12" t="s">
-        <v>72</v>
+        <v>84</v>
       </c>
       <c r="N10" s="12" t="s">
-        <v>73</v>
+        <v>85</v>
       </c>
       <c r="O10" s="12" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
+        <v>86</v>
+      </c>
+      <c r="P10" s="12" t="s">
+        <v>86</v>
+      </c>
+      <c r="Q10" s="12" t="s">
+        <v>86</v>
+      </c>
+      <c r="R10" s="12" t="s">
+        <v>86</v>
+      </c>
+      <c r="S10" s="12" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="11" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A11" s="13"/>
       <c r="B11" s="13"/>
       <c r="C11" s="13"/>
@@ -1217,8 +1324,12 @@
       <c r="M11" s="13"/>
       <c r="N11" s="13"/>
       <c r="O11" s="13"/>
-    </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P11" s="13"/>
+      <c r="Q11" s="13"/>
+      <c r="R11" s="13"/>
+      <c r="S11" s="13"/>
+    </row>
+    <row r="12" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A12" s="13"/>
       <c r="B12" s="13"/>
       <c r="C12" s="13"/>
@@ -1234,8 +1345,12 @@
       <c r="M12" s="13"/>
       <c r="N12" s="13"/>
       <c r="O12" s="13"/>
-    </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P12" s="13"/>
+      <c r="Q12" s="13"/>
+      <c r="R12" s="13"/>
+      <c r="S12" s="13"/>
+    </row>
+    <row r="13" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A13" s="13"/>
       <c r="B13" s="13"/>
       <c r="C13" s="13"/>
@@ -1251,8 +1366,12 @@
       <c r="M13" s="13"/>
       <c r="N13" s="13"/>
       <c r="O13" s="13"/>
-    </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P13" s="13"/>
+      <c r="Q13" s="13"/>
+      <c r="R13" s="13"/>
+      <c r="S13" s="13"/>
+    </row>
+    <row r="14" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A14" s="13"/>
       <c r="B14" s="13"/>
       <c r="C14" s="13"/>
@@ -1268,8 +1387,12 @@
       <c r="M14" s="13"/>
       <c r="N14" s="13"/>
       <c r="O14" s="13"/>
-    </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P14" s="13"/>
+      <c r="Q14" s="13"/>
+      <c r="R14" s="13"/>
+      <c r="S14" s="13"/>
+    </row>
+    <row r="15" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A15" s="13"/>
       <c r="B15" s="13"/>
       <c r="C15" s="13"/>
@@ -1285,8 +1408,12 @@
       <c r="M15" s="13"/>
       <c r="N15" s="13"/>
       <c r="O15" s="13"/>
-    </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P15" s="13"/>
+      <c r="Q15" s="13"/>
+      <c r="R15" s="13"/>
+      <c r="S15" s="13"/>
+    </row>
+    <row r="16" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A16" s="13"/>
       <c r="B16" s="13"/>
       <c r="C16" s="13"/>
@@ -1302,8 +1429,12 @@
       <c r="M16" s="13"/>
       <c r="N16" s="13"/>
       <c r="O16" s="13"/>
-    </row>
-    <row r="17" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P16" s="13"/>
+      <c r="Q16" s="13"/>
+      <c r="R16" s="13"/>
+      <c r="S16" s="13"/>
+    </row>
+    <row r="17" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A17" s="13"/>
       <c r="B17" s="13"/>
       <c r="C17" s="13"/>
@@ -1319,8 +1450,12 @@
       <c r="M17" s="13"/>
       <c r="N17" s="13"/>
       <c r="O17" s="13"/>
-    </row>
-    <row r="18" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P17" s="13"/>
+      <c r="Q17" s="13"/>
+      <c r="R17" s="13"/>
+      <c r="S17" s="13"/>
+    </row>
+    <row r="18" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A18" s="13"/>
       <c r="B18" s="13"/>
       <c r="C18" s="13"/>
@@ -1336,8 +1471,12 @@
       <c r="M18" s="13"/>
       <c r="N18" s="13"/>
       <c r="O18" s="13"/>
-    </row>
-    <row r="19" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P18" s="13"/>
+      <c r="Q18" s="13"/>
+      <c r="R18" s="13"/>
+      <c r="S18" s="13"/>
+    </row>
+    <row r="19" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A19" s="13"/>
       <c r="B19" s="13"/>
       <c r="C19" s="13"/>
@@ -1353,8 +1492,12 @@
       <c r="M19" s="13"/>
       <c r="N19" s="13"/>
       <c r="O19" s="13"/>
-    </row>
-    <row r="20" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P19" s="13"/>
+      <c r="Q19" s="13"/>
+      <c r="R19" s="13"/>
+      <c r="S19" s="13"/>
+    </row>
+    <row r="20" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A20" s="13"/>
       <c r="B20" s="13"/>
       <c r="C20" s="13"/>
@@ -1370,8 +1513,12 @@
       <c r="M20" s="13"/>
       <c r="N20" s="13"/>
       <c r="O20" s="13"/>
-    </row>
-    <row r="21" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P20" s="13"/>
+      <c r="Q20" s="13"/>
+      <c r="R20" s="13"/>
+      <c r="S20" s="13"/>
+    </row>
+    <row r="21" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A21" s="13"/>
       <c r="B21" s="13"/>
       <c r="C21" s="13"/>
@@ -1387,8 +1534,12 @@
       <c r="M21" s="13"/>
       <c r="N21" s="13"/>
       <c r="O21" s="13"/>
-    </row>
-    <row r="22" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P21" s="13"/>
+      <c r="Q21" s="13"/>
+      <c r="R21" s="13"/>
+      <c r="S21" s="13"/>
+    </row>
+    <row r="22" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A22" s="13"/>
       <c r="B22" s="13"/>
       <c r="C22" s="13"/>
@@ -1404,8 +1555,12 @@
       <c r="M22" s="13"/>
       <c r="N22" s="13"/>
       <c r="O22" s="13"/>
-    </row>
-    <row r="23" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P22" s="13"/>
+      <c r="Q22" s="13"/>
+      <c r="R22" s="13"/>
+      <c r="S22" s="13"/>
+    </row>
+    <row r="23" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A23" s="13"/>
       <c r="B23" s="13"/>
       <c r="C23" s="13"/>
@@ -1421,8 +1576,12 @@
       <c r="M23" s="13"/>
       <c r="N23" s="13"/>
       <c r="O23" s="13"/>
-    </row>
-    <row r="24" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P23" s="13"/>
+      <c r="Q23" s="13"/>
+      <c r="R23" s="13"/>
+      <c r="S23" s="13"/>
+    </row>
+    <row r="24" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A24" s="13"/>
       <c r="B24" s="13"/>
       <c r="C24" s="13"/>
@@ -1438,8 +1597,12 @@
       <c r="M24" s="13"/>
       <c r="N24" s="13"/>
       <c r="O24" s="13"/>
-    </row>
-    <row r="25" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P24" s="13"/>
+      <c r="Q24" s="13"/>
+      <c r="R24" s="13"/>
+      <c r="S24" s="13"/>
+    </row>
+    <row r="25" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A25" s="13"/>
       <c r="B25" s="13"/>
       <c r="C25" s="13"/>
@@ -1455,8 +1618,12 @@
       <c r="M25" s="13"/>
       <c r="N25" s="13"/>
       <c r="O25" s="13"/>
-    </row>
-    <row r="26" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P25" s="13"/>
+      <c r="Q25" s="13"/>
+      <c r="R25" s="13"/>
+      <c r="S25" s="13"/>
+    </row>
+    <row r="26" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A26" s="13"/>
       <c r="B26" s="13"/>
       <c r="C26" s="13"/>
@@ -1472,8 +1639,12 @@
       <c r="M26" s="13"/>
       <c r="N26" s="13"/>
       <c r="O26" s="13"/>
-    </row>
-    <row r="27" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P26" s="13"/>
+      <c r="Q26" s="13"/>
+      <c r="R26" s="13"/>
+      <c r="S26" s="13"/>
+    </row>
+    <row r="27" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A27" s="13"/>
       <c r="B27" s="13"/>
       <c r="C27" s="13"/>
@@ -1489,8 +1660,12 @@
       <c r="M27" s="13"/>
       <c r="N27" s="13"/>
       <c r="O27" s="13"/>
-    </row>
-    <row r="28" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P27" s="13"/>
+      <c r="Q27" s="13"/>
+      <c r="R27" s="13"/>
+      <c r="S27" s="13"/>
+    </row>
+    <row r="28" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A28" s="13"/>
       <c r="B28" s="13"/>
       <c r="C28" s="13"/>
@@ -1506,8 +1681,12 @@
       <c r="M28" s="13"/>
       <c r="N28" s="13"/>
       <c r="O28" s="13"/>
-    </row>
-    <row r="29" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P28" s="13"/>
+      <c r="Q28" s="13"/>
+      <c r="R28" s="13"/>
+      <c r="S28" s="13"/>
+    </row>
+    <row r="29" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A29" s="13"/>
       <c r="B29" s="13"/>
       <c r="C29" s="13"/>
@@ -1523,8 +1702,12 @@
       <c r="M29" s="13"/>
       <c r="N29" s="13"/>
       <c r="O29" s="13"/>
-    </row>
-    <row r="30" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P29" s="13"/>
+      <c r="Q29" s="13"/>
+      <c r="R29" s="13"/>
+      <c r="S29" s="13"/>
+    </row>
+    <row r="30" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A30" s="13"/>
       <c r="B30" s="13"/>
       <c r="C30" s="13"/>
@@ -1540,13 +1723,17 @@
       <c r="M30" s="13"/>
       <c r="N30" s="13"/>
       <c r="O30" s="13"/>
+      <c r="P30" s="13"/>
+      <c r="Q30" s="13"/>
+      <c r="R30" s="13"/>
+      <c r="S30" s="13"/>
     </row>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="A1:O2"/>
+    <mergeCell ref="A1:S2"/>
     <mergeCell ref="A4:D5"/>
-    <mergeCell ref="E4:J5"/>
-    <mergeCell ref="K4:O5"/>
+    <mergeCell ref="E4:N5"/>
+    <mergeCell ref="O4:S5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>